<commit_message>
scan: seg8 2026-06-23 01:13 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq0_2026-06-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>69.59558877195705</v>
+        <v>69.59558877059362</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>40.86008539207342</v>
+        <v>40.86008538307081</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.853244380446803</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.3801788229875056</v>
+        <v>0.3801788230184169</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>64.55856296414979</v>
+        <v>64.55856295378577</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>25.64112782660538</v>
+        <v>25.64112769316916</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.969068540860017</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.2099741532307587</v>
+        <v>0.2099741534574154</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>65.67368618835644</v>
+        <v>65.67368618109188</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>28.45971020149237</v>
+        <v>28.45971018133653</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.8771660056827324</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.6087907262639423</v>
+        <v>0.6087907263360677</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1124.569102553254</v>
+        <v>1124.569102553244</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>31.25</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>66.15479890053379</v>
+        <v>66.15479822919615</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>23.84481660199638</v>
+        <v>23.8448166707275</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.255789944104196</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1594615942954637</v>
+        <v>0.1594615952536349</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>65.87947983257928</v>
+        <v>65.87947973580276</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>11.82370213313866</v>
+        <v>11.82370214877799</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.406880414820684</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.8354972616887342</v>
+        <v>0.8354972618329672</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>61.45124388974835</v>
+        <v>61.45124389190117</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>35.38041322065952</v>
+        <v>35.38041314105026</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.238665692297571</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.4506237725960265</v>
+        <v>0.4506237726990569</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>76.93553142159037</v>
+        <v>76.93553140119582</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>48.08064345290865</v>
+        <v>48.08064346052839</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.57275848944979</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.9881619325802936</v>
+        <v>0.9881619326730164</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1003.980693423682</v>
+        <v>1003.980693423683</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>51.9</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>70.96283699608477</v>
+        <v>70.9628368965917</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>17.78960403708079</v>
+        <v>17.78960397437504</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>3.471617642284939</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.1168343974483931</v>
+        <v>0.1168343981695952</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>75.71784123715949</v>
+        <v>75.71784123143161</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>29.61719451434673</v>
+        <v>29.6171944588962</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.209387368569256</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>4.891199226346973</v>
+        <v>4.891199226862129</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>62.65697725922002</v>
+        <v>62.65697725080676</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>19.43262630212842</v>
+        <v>19.43262623524666</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.022553631580065</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.2685194906373966</v>
+        <v>0.2685194906580033</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63.83144590298788</v>
+        <v>63.8314458942391</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>16.82304847681699</v>
+        <v>16.82304839128533</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.608876466053075</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.6784237801493451</v>
+        <v>0.6784237802214577</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64.1579346175904</v>
+        <v>64.15793444795364</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>26.17749355997542</v>
+        <v>26.17749378920361</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>2.043089499970447</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.018382296949146</v>
+        <v>0.0183822973818679</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>68.58642003791871</v>
+        <v>68.58641999089885</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>41.91956274572706</v>
+        <v>41.91956294853944</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.135532437526354</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.0548874223316899</v>
+        <v>0.0548874224347191</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>68.98409313463483</v>
+        <v>68.98409312333742</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>22.63461045578711</v>
+        <v>22.63461045108226</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.9835198283376672</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>44.6147284181288</v>
+        <v>44.61472841957108</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72.97927226338979</v>
+        <v>72.97927221255981</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>45.08161635725729</v>
+        <v>45.08161646104636</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.9938149242520528</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>2.150895658459309</v>
+        <v>2.15089565953081</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>64.49497009935682</v>
+        <v>64.49497004774815</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>26.72938822014681</v>
+        <v>26.72938825864924</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.9561264018893468</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.6001407662871938</v>
+        <v>0.6001407664932588</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>64.42835926354329</v>
+        <v>64.42835922889549</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>36.3035513665844</v>
+        <v>36.30355113262873</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.197439490609342</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.9626376768668958</v>
+        <v>-0.9626376762693436</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>57.51831253722471</v>
+        <v>57.51831249514851</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>19.82871407854998</v>
+        <v>19.82871407854999</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.199061055953782</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.3495696757906606</v>
+        <v>0.3495696758009674</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>75.35275300420371</v>
+        <v>75.35275299110876</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>39.7546257792641</v>
+        <v>39.7546257089362</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.1383122787513019</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>4.537360015799598</v>
+        <v>4.537360016067467</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>65.58182995836191</v>
+        <v>65.58182991487961</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>45.38611293677669</v>
+        <v>45.38611277925734</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9431597474875156</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.5889117443605256</v>
+        <v>0.588911744504764</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>62.2314229926995</v>
+        <v>62.23142298842679</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>15.70401930386237</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1.940616800784702</v>
+        <v>1.940616801093755</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>61.16625033657416</v>
+        <v>61.16625031388531</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>31.78908805066253</v>
+        <v>31.78908802916535</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.643165579181209</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.0073584655692324</v>
+        <v>0.0073584657237717</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>72.46923038270708</v>
+        <v>72.46923027440204</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>49.66176198138334</v>
+        <v>49.66176193376251</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.9942924548471482</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0642099503682325</v>
+        <v>0.0642099505536797</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.25926522949772</v>
+        <v>57.25926520840996</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>28.01148894075989</v>
+        <v>28.01148899744418</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.7822310450952619</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0673104849856743</v>
+        <v>0.0673104850165846</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>70.25998963441131</v>
+        <v>70.25998961844782</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>52.29333003237685</v>
+        <v>52.29332999921274</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.5280890818377724</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.1493520363925879</v>
+        <v>0.1493520365265244</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>791.9667700270419</v>
+        <v>791.966770027042</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>68.5</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>64.23671819305181</v>
+        <v>64.23671812308788</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>26.36423427612994</v>
+        <v>26.36423421544531</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.424886942503179</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.5287914096159914</v>
+        <v>0.5287914097190241</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>67.41419827326625</v>
+        <v>67.41419827077718</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>24.38878899776504</v>
+        <v>24.38878893728421</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>2.959084355870412</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>3.887979922626279</v>
+        <v>3.887979922822041</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63.71430680468519</v>
+        <v>63.71430679984179</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>52.47517685687641</v>
+        <v>52.47517687639044</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.3281065223729457</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.1931520533933053</v>
+        <v>-0.1931520534036082</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>58.06254140262515</v>
+        <v>58.06254139827304</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15.82779263824517</v>
+        <v>15.82779263397188</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.924707423289001</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.9006470399331372</v>
+        <v>0.9006470399743549</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>86.88445936337443</v>
+        <v>86.88445933861206</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>47.77952041912421</v>
+        <v>47.77952042384664</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>3.295189029465377</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.6326324696591328</v>
+        <v>0.6326324697003433</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>57.2653514399119</v>
+        <v>57.26535143082394</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>22.1824198347704</v>
+        <v>22.18241978948286</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.8049930117603062</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.5015422613556892</v>
+        <v>0.5015422610466194</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46.5960435368748</v>
+        <v>46.59604348274354</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22.01550476584379</v>
+        <v>22.01550484399795</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>2.33958811238229</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.4895502471901019</v>
+        <v>0.4895502474373725</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.25405517168402</v>
+        <v>57.25405517479754</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>28.04075816042352</v>
+        <v>28.04075820912518</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.6354795163046555</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.5862013593110147</v>
+        <v>-0.5862013592389062</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>64.01813011294725</v>
+        <v>64.01813002978358</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>25.8835923803235</v>
+        <v>25.88359258951458</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.373160299025048</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.0789216307338719</v>
+        <v>0.0789216308472004</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>59.33547491343495</v>
+        <v>59.33547490604139</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>30.84352330423118</v>
+        <v>30.84352329306955</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.7699492760310126</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0863986467048911</v>
+        <v>-0.08639864670076949</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>59.99794027384712</v>
+        <v>59.99794023164745</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>35.68425757555578</v>
+        <v>35.68425754254921</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5579440142095334</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.7162995092321971</v>
+        <v>-0.7162995090673485</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>58.11177563596416</v>
+        <v>58.11177563903534</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>45.98977109207414</v>
+        <v>45.9897711065934</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.6270715116604564</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.1959309677291622</v>
+        <v>-0.1959309677353433</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>52.8054275190024</v>
+        <v>52.80542741835687</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>21.40231525481962</v>
+        <v>21.40231525280837</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.509018768003842</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.1895131967770338</v>
+        <v>-0.1895131966740026</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.80818501797327</v>
+        <v>54.80818490388685</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>42.39557116368682</v>
+        <v>42.3955713459255</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.3821624607517451</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.7368359409478553</v>
+        <v>-0.7368359405563378</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>57.54622170988952</v>
+        <v>57.54622167005932</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>18.13437269347849</v>
+        <v>18.13437249318698</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.6814877443594275</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>3.293514962227169</v>
+        <v>3.293514963257401</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>56.65470415525528</v>
+        <v>56.6547039151308</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.12225372055783</v>
+        <v>27.12225388015392</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.8991745258083679</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.0006743080032375999</v>
+        <v>-0.0006743076735413</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>50.83616307661456</v>
+        <v>50.83616303318286</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>23.04419664105085</v>
+        <v>23.04419673227775</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.794419155917807</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-2.730973987394464</v>
+        <v>-2.730973986776283</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>614.1144005986504</v>
+        <v>614.1144005986505</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>2580</v>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>56.95794920830301</v>
+        <v>56.95794920503545</v>
       </c>
       <c r="I44" s="2" t="n">
         <v>15.5477678051129</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-6.10649737184265</v>
+        <v>-6.106497370709107</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>63.86411652743199</v>
+        <v>63.8641164770158</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>28.52109500677883</v>
+        <v>28.52109513317729</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8369877124567728</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.1272129545436153</v>
+        <v>0.1272129545230091</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>51.94648343063086</v>
+        <v>51.94648340484858</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>26.14499218215988</v>
+        <v>26.14499212133084</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.669419568313676</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.661705646078607</v>
+        <v>-1.661705645996184</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>52.83183261322618</v>
+        <v>52.83183399978737</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>26.5814810037813</v>
+        <v>26.58148143844532</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.2077492333146421</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.7525049509666646</v>
+        <v>-0.7525049563241781</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>55.83387052409307</v>
+        <v>55.83387046532816</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>16.24854468581634</v>
+        <v>16.24854469955455</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.172890082970546</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.105386604661611</v>
+        <v>0.1053866046307024</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>54.90300655815783</v>
+        <v>54.90300655359036</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>27.55141348642664</v>
+        <v>27.5514134586565</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.3618269546689292</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.1519155199946853</v>
+        <v>-0.1519155199431674</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>53.64615254410147</v>
+        <v>53.64615253493402</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>30.14725035967296</v>
+        <v>30.14725024698082</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.2971606409080504</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.142772357722809</v>
+        <v>-1.1427723576713</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>50.57283531423098</v>
+        <v>50.57283527072747</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>23.49898172952779</v>
+        <v>23.49898172740304</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.7346651641210479</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-3.057475030758992</v>
+        <v>-3.057475031789253</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>51.26560522295623</v>
+        <v>51.26559700310184</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.23807721429901</v>
+        <v>22.23807741342041</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.1499514345332174</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0071905713369371</v>
+        <v>0.0071905737787265</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>57.32267030322254</v>
+        <v>57.32267014448656</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>41.90835752582685</v>
+        <v>41.90835798909784</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.017511383441774</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5321370781774939</v>
+        <v>0.5321370789811188</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>54.98631658364435</v>
+        <v>54.9863165815282</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>11.36022502801612</v>
+        <v>11.36022502379912</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.474964807338702</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.3723851006035327</v>
+        <v>0.3723851006138314</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.51964995590186</v>
+        <v>52.51964992259449</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.81611235904887</v>
+        <v>11.8161123498208</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.753207679469957</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0344693147421569</v>
+        <v>0.0344693147936721</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>53.35009989293047</v>
+        <v>53.35009989511743</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>8.400400934541478</v>
+        <v>8.400400795268519</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.192298343248257</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.445792757370358</v>
+        <v>0.4457927575645901</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>47.67482509978447</v>
+        <v>47.67482517476118</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>18.28256908656216</v>
+        <v>18.28256913454973</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.298057444164708</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-1.288138017698971</v>
+        <v>-1.288138016730508</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>50.63977864058948</v>
+        <v>50.63977881356394</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22.35904751275794</v>
+        <v>22.3590474504508</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>2.260824998587477</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>50.11317407492659</v>
+        <v>50.11317405888905</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.46771583009723</v>
+        <v>20.46771579075914</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.7648356967119617</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-17.43978744029621</v>
+        <v>-17.43978743875062</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>488.4477837682083</v>
+        <v>488.4477837682082</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>21</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>55.46267582435435</v>
+        <v>55.46267573307806</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>17.35623868896336</v>
+        <v>17.35623874010133</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.7063279983544034</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0605887285028038</v>
+        <v>0.0605887285131106</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>53.51188688040001</v>
+        <v>53.51188688549981</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.06118588154812</v>
+        <v>11.06118586677728</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.6830432086685755</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.6697082405622794</v>
+        <v>-0.6697082405416896</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>54.87452164948149</v>
+        <v>54.87452151573555</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.361986100811</v>
+        <v>16.3619861477089</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.7614981024014497</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0693246910294105</v>
+        <v>0.0693246913825583</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>28.27555273020444</v>
+        <v>28.27555276617929</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.29967226429201</v>
+        <v>23.29967230730791</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1.924124893198958</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.0051653699512643</v>
+        <v>-0.0051653699718711</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>55.89061040156938</v>
+        <v>55.89061018749504</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>18.38764624417525</v>
+        <v>18.38764637365991</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.061997501976454</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>3.567369518038106</v>
+        <v>3.567369520819929</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>55.74733215209982</v>
+        <v>55.74733213699414</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>12.04049587188776</v>
+        <v>12.04049589925991</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.519241872689839</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.1333834152612707</v>
+        <v>0.1333834153849077</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>52.29169889183252</v>
+        <v>52.29169873653724</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>22.51199716531903</v>
+        <v>22.51199739479586</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.435078386742027</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0141075564905358</v>
+        <v>-0.0141075564081129</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>432.630409445486</v>
+        <v>432.6304094454487</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>36.9</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>55.38582440852187</v>
+        <v>55.38582422030684</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>13.39283647760869</v>
+        <v>13.39283646596866</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1.849682356257207</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0579437955005494</v>
+        <v>0.0579437955211589</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>428.2843510827441</v>
+        <v>428.284351082744</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>30.85</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>44.86990860353266</v>
+        <v>44.86990859424216</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>21.88838538618687</v>
+        <v>21.88838548255623</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5467728622981183</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.9646113947606968</v>
+        <v>-0.9646113947812996</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>47.18393826152934</v>
+        <v>47.18393819854057</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>16.37289820071432</v>
+        <v>16.3728981958836</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.5390654364518265</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.2519479784929129</v>
+        <v>-0.2519479782662535</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>53.39087740343192</v>
+        <v>53.39087736386375</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>27.44137324390826</v>
+        <v>27.44137325140576</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.394384519624956</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.3206986549324043</v>
+        <v>-0.3206986548705872</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>45.27220691551383</v>
+        <v>45.27220636238286</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>9.117409637206441</v>
+        <v>9.117409714563278</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.7593349520331367</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.0028730132842541</v>
+        <v>0.0028730134387985</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.93579557266403</v>
+        <v>41.93579559192604</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>24.40531162064339</v>
+        <v>24.40531154139332</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.6434431797890061</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-1.355645284331899</v>
+        <v>-1.355645283713735</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>48.06059120480347</v>
+        <v>48.06059119249452</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.01325526438995</v>
+        <v>15.01325527536611</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.3614776128228654</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>51.40893070150225</v>
+        <v>51.4089306625831</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.17571971725771</v>
+        <v>14.17571973192748</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.266102507295338</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0019790874677654</v>
+        <v>0.0019790875501843</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>44.04237382303968</v>
+        <v>44.04237337502833</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>25.03097912373814</v>
+        <v>25.03097939186872</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.191885049357884</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0010938467836872</v>
+        <v>-0.0010938466930211</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>44.82269501195421</v>
+        <v>44.82269502083291</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>15.3234365588359</v>
+        <v>15.32343663776853</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5488191355136035</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.2174962681478882</v>
+        <v>-0.2174962682200105</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>51.24354699722731</v>
+        <v>51.24354695247745</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>16.79279551782102</v>
+        <v>16.79279549981724</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>2.088602123471383</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.0012368219812872</v>
+        <v>-0.0012368218061353</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>380.4322713499453</v>
+        <v>380.4322713499452</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>33.1</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>54.39471133932904</v>
+        <v>54.39471126577049</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.9162150105544</v>
+        <v>13.916215073479</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.566637085314575</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.2089195811398557</v>
+        <v>0.208919581242887</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>46.2363472515177</v>
+        <v>46.23634738732677</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>31.22300264704201</v>
+        <v>31.22300270068158</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.3598438101892344</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.07328776115507681</v>
+        <v>-0.0732877611385917</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>375.6574954354653</v>
+        <v>375.6574954354973</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>13.75</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>45.69919124781971</v>
+        <v>45.69919107208833</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>13.78650531663379</v>
+        <v>13.78650537656794</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.5644699795102748</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0054382791767491</v>
+        <v>0.0054382792385649</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>44.66159507505788</v>
+        <v>44.66159509068054</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>19.48198900769686</v>
+        <v>19.48198909021259</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.7169608095021641</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.2624294674933219</v>
+        <v>-0.2624294673902918</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>50.68732582579276</v>
+        <v>50.68732579016481</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>6.426530978227574</v>
+        <v>6.42653117795351</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.7792293186733704</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.1518410278392454</v>
+        <v>-0.1518410278083356</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>45.59761393266653</v>
+        <v>45.59761390193996</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>26.61827319294668</v>
+        <v>26.61827329868101</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.9685422225323908</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-3.572183018249115</v>
+        <v>-3.572183017836993</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>41.87734973265555</v>
+        <v>41.87734983758553</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>23.03334672436788</v>
+        <v>23.03334679726172</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.520003901614293</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.0690101961545381</v>
+        <v>0.0690101962163521</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>349.2180397650946</v>
+        <v>349.2180397650944</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>20.8</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.26407578055966</v>
+        <v>49.26407482883941</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>34.4405674189208</v>
+        <v>34.44056778541745</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.6646850181594461</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0712526725198778</v>
+        <v>0.0712526737768321</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>48.01337869044994</v>
+        <v>48.01337871956068</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>34.3705367576272</v>
+        <v>34.3705367273507</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.6698915095888113</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.28717673551696</v>
+        <v>48.28717668369411</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>54.5933361099236</v>
+        <v>54.59333606315741</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.874212610841705</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0281975007191715</v>
+        <v>0.0281975007294745</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>54.89931329316885</v>
+        <v>54.89931288876718</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>16.05993059705318</v>
+        <v>16.05993068974259</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.8549612538726895</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0443917998389766</v>
+        <v>0.0443917998904898</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.89451078492315</v>
+        <v>42.89451066711559</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>22.09680395257257</v>
+        <v>22.09680394781921</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.009250482893613</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0112675829195562</v>
+        <v>0.0112675829710731</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.18854533997536</v>
+        <v>44.18854528499001</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>20.66452749592273</v>
+        <v>20.66452755838376</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.4189688655753164</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.4487386973283707</v>
+        <v>-0.4487386969399045</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>335.2650917339703</v>
+        <v>335.2650917339828</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>48.35</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>51.68098153522982</v>
+        <v>51.68098151820458</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>7.720185033250349</v>
+        <v>7.720185076888203</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.106490511414517</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-1.121995149580545</v>
+        <v>-1.121995149189037</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>48.23761820726137</v>
+        <v>48.23761820605029</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>19.88053374435624</v>
+        <v>19.8805337193958</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.7458438028428901</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.262957764848092</v>
+        <v>-2.262957764745047</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>42.53585389857169</v>
+        <v>42.53585375597746</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>15.77899461616967</v>
+        <v>15.77899460888599</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.4313170870680718</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.3113432794012227</v>
+        <v>-0.3113432787830521</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>53.8208523386947</v>
+        <v>53.82085229956334</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.86933979750362</v>
+        <v>16.86933979891073</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.7760868196681455</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.9626268712581948</v>
+        <v>0.9626268712994142</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>46.57420938072929</v>
+        <v>46.57420924828515</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>20.11227722877092</v>
+        <v>20.11227765165689</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.1811762536410148</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0029937845322541</v>
+        <v>0.0029937846661928</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.2655719812246</v>
+        <v>49.26557208232486</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>12.66405181098009</v>
+        <v>12.6640518415479</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.3172736015320926</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0137438361062598</v>
+        <v>0.0137438360650481</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>50.51326472259954</v>
+        <v>50.51326469424898</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>17.04218168405697</v>
+        <v>17.04218167038091</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4824714651758677</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>1.592864857436546</v>
+        <v>1.592864858260781</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.88195784930714</v>
+        <v>42.88195787726519</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>21.12994765596171</v>
+        <v>21.12994758004963</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4438394880211547</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-1.484672549799926</v>
+        <v>-1.484672549676292</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>49.87340294324632</v>
+        <v>49.87340282988498</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>18.30969735047054</v>
+        <v>18.30969736426349</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.3554019346876853</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.1796859043720784</v>
+        <v>-0.1796859041866238</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>46.93571453569233</v>
+        <v>46.93571449964211</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.27249480085161</v>
+        <v>14.2724947911344</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.8170877346675346</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0640434823103562</v>
+        <v>0.0640434823000549</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>47.39732733479372</v>
+        <v>47.39732707233407</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>16.58992181365726</v>
+        <v>16.58992203622394</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.081620368932414</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0335369438129198</v>
+        <v>0.033536944049887</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>256.1867504647509</v>
+        <v>256.1867504647508</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>56.9</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>39.54698772886026</v>
+        <v>39.54698741100519</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>27.72932161994437</v>
+        <v>27.72932142599461</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.7189856482554586</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.332474538329754</v>
+        <v>-0.3324745374230979</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>37.06069224143736</v>
+        <v>37.06069238309136</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.6947604376487</v>
+        <v>16.69476043135234</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>1.756846082439818</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.1635551549153128</v>
+        <v>-0.1635551551213642</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,7 +5958,7 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>47.23998428707663</v>
+        <v>47.23998423092257</v>
       </c>
       <c r="I104" s="2" t="n">
         <v>44.93382172741092</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0519444059509916</v>
+        <v>0.051944406033418</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.64636116007859</v>
+        <v>42.64636135187907</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.27091364114954</v>
+        <v>15.270913803915</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.586095535055095</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1160713945523277</v>
+        <v>-0.116071394325668</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>41.87597256488181</v>
+        <v>41.87597227500446</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.70723994917432</v>
+        <v>13.70724001373154</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7098659574734414</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0364865680846615</v>
+        <v>-0.0364865679198157</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>202.6641450050433</v>
+        <v>202.6641450050428</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>75.8</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>42.70053484201752</v>
+        <v>42.70053452550619</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>13.3142916396753</v>
+        <v>13.31429180582463</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5371818650358262</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.2076337971571348</v>
+        <v>-0.2076337958589686</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>168.6298885805149</v>
+        <v>168.6298885805145</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>65.5</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>47.33473588092828</v>
+        <v>47.33473562324552</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.62608979137409</v>
+        <v>17.62608984131542</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6560198111571076</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.4801197808250285</v>
+        <v>-0.4801197793414167</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>50.076709984186</v>
+        <v>50.07670991294149</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.00529683981106</v>
+        <v>15.00529675219222</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.6009081782068267</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.327992282955595</v>
+        <v>-0.3279922824258769</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>48.09128771253064</v>
+        <v>48.09128754768817</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.10261260835905</v>
+        <v>21.10261274911135</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.3840277026573738</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0240128290813063</v>
+        <v>-0.0240128289267618</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>33.61177959099254</v>
+        <v>33.61177961229342</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.65099479352688</v>
+        <v>18.65099493266558</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.6381631262192017</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.2325050045260416</v>
+        <v>-0.2325050043921024</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.8600433568771</v>
+        <v>44.86004343903732</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>13.17613251640999</v>
+        <v>13.17613259181264</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.6004335764880752</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1210145387589595</v>
+        <v>-0.121014538614719</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>127.8713457439768</v>
+        <v>127.8713457439767</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>33.15</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>37.70635937767079</v>
+        <v>37.70635924009818</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>21.65230639401056</v>
+        <v>21.65230643254071</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.5948457930170534</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1053903127947737</v>
+        <v>-0.1053903127329569</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>34.97044056295354</v>
+        <v>34.97044051574122</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.03814674351924</v>
+        <v>17.03814672925639</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.03702320428652</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.2140993961644114</v>
+        <v>-0.2140993961335042</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>114.1955976636101</v>
+        <v>114.19559766361</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>21.45</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.90699899727415</v>
+        <v>40.90699867112777</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>13.2906902500732</v>
+        <v>13.29069036268916</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.244948880802941</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.020727103951219</v>
+        <v>-0.0207271037966756</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>103.1287326571103</v>
+        <v>103.1287326571105</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>22</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.56768926105656</v>
+        <v>43.56768908213066</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>18.14044074335382</v>
+        <v>18.14044108100936</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.6688326619376526</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2442732867573109</v>
+        <v>-0.2442732865512517</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>

</xml_diff>